<commit_message>
Actualización para reintentos en QR y subida de Excel desde el front al back.
</commit_message>
<xml_diff>
--- a/input/Producción factura C/Facturacion.xlsx
+++ b/input/Producción factura C/Facturacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programación\trabajo\Facturación Electronica Python\InvoicerPRO-Development\input\Factura C\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\InvoicePRO\invoice-pro-back-local\input\Factura C\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C2D6E7-DAF3-4107-BA6C-F2450C5CBF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFFDFCB9-FCBF-4D8E-BB6C-2FD7FD6C827E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4245" yWindow="4485" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Factura C" sheetId="1" r:id="rId1"/>
@@ -143,7 +143,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -454,7 +454,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -885,7 +885,7 @@
         <v>33</v>
       </c>
       <c r="B2" s="33">
-        <v>46041</v>
+        <v>46056</v>
       </c>
       <c r="C2" s="33">
         <v>45505</v>

</xml_diff>